<commit_message>
Update DRC files to rename 'MEAS' to 'PTECT' and enhance error handling for prohibited areas
</commit_message>
<xml_diff>
--- a/Document/TR-1um_GDSII_Table.xlsx
+++ b/Document/TR-1um_GDSII_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Library/CloudStorage/Dropbox/91_OpenPDK/TR-1um/Document/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB07B079-2974-9842-AB36-D3B33B28C33E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A104E4FE-DCA7-2F42-9960-2912C2BC6BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="840" yWindow="760" windowWidth="29400" windowHeight="18600" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
@@ -308,9 +308,6 @@
     <t>M1 Pin</t>
   </si>
   <si>
-    <t>SCRIBE</t>
-  </si>
-  <si>
     <t>Waiver region (EDGE SEAL)</t>
   </si>
   <si>
@@ -326,12 +323,6 @@
     <t>Active for resistor</t>
   </si>
   <si>
-    <t>MEAS</t>
-  </si>
-  <si>
-    <t>Measurement region</t>
-  </si>
-  <si>
     <t>GC</t>
   </si>
   <si>
@@ -345,6 +336,15 @@
   </si>
   <si>
     <t>PO</t>
+  </si>
+  <si>
+    <t>SCRB</t>
+  </si>
+  <si>
+    <t>PTECT</t>
+  </si>
+  <si>
+    <t>Protect region (LOGO)</t>
   </si>
 </sst>
 </file>
@@ -1439,7 +1439,7 @@
         <v>3</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M10" s="5"/>
     </row>
@@ -1700,7 +1700,7 @@
       <c r="C22" s="12"/>
       <c r="E22" s="15"/>
       <c r="G22" s="12" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H22" s="1">
         <v>8</v>
@@ -1709,7 +1709,7 @@
         <v>1</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="M22" s="5"/>
     </row>
@@ -1718,7 +1718,7 @@
       <c r="C23" s="12"/>
       <c r="E23" s="15"/>
       <c r="G23" s="12" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="H23" s="1">
         <v>8</v>
@@ -1727,7 +1727,7 @@
         <v>2</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="M23" s="5"/>
     </row>
@@ -1961,7 +1961,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="12" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="H33" s="1">
         <v>14</v>
@@ -2094,7 +2094,7 @@
     <row r="39" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B39" s="54"/>
       <c r="C39" s="55" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D39" s="56">
         <v>63</v>
@@ -2104,7 +2104,7 @@
       </c>
       <c r="F39" s="56"/>
       <c r="G39" s="55" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="H39" s="56">
         <v>63</v>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="J39" s="56"/>
       <c r="K39" s="58" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="L39" s="56"/>
       <c r="M39" s="59"/>
@@ -2122,7 +2122,7 @@
     <row r="40" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B40" s="54"/>
       <c r="C40" s="55" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="D40" s="56">
         <v>80</v>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="F40" s="56"/>
       <c r="G40" s="55" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="H40" s="56">
         <v>80</v>
@@ -2142,7 +2142,7 @@
       </c>
       <c r="J40" s="56"/>
       <c r="K40" s="58" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="L40" s="56"/>
       <c r="M40" s="59"/>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="L45" s="21"/>
       <c r="M45" s="62" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="46" spans="2:13" x14ac:dyDescent="0.2">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="L46" s="6"/>
       <c r="M46" s="60" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="47" spans="2:13" x14ac:dyDescent="0.2">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="L47" s="6"/>
       <c r="M47" s="60" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.2">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="L48" s="6"/>
       <c r="M48" s="60" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="49" spans="2:13" x14ac:dyDescent="0.2">
@@ -2674,12 +2674,12 @@
         <v>80</v>
       </c>
       <c r="C66" s="61" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="67" spans="2:3" s="2" customFormat="1" ht="19" x14ac:dyDescent="0.2">
       <c r="C67" s="61" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>